<commit_message>
Switch searcher to API-based session flow
Major refactor of searcher.py to use an API-based approach instead of browser-only scraping: login once via browser to extract cookies, build a requests.Session (including x-xsrf-token header), reuse/save/delete session cookies (session_cookies.pkl), and perform report searches by POSTing to the SEARCH_API_URL with 2Captcha token. Added cookie extraction, session validation, and automatic OTP handling (polls a Google Sheet cell for user-provided code). Updated solve_recaptcha to submit/poll 2Captcha and added debug logging for API calls. Also updated config.py with a new CAPTCHA_SITE_KEY, bumped progress.txt, and included an updated crash_reports.xlsx and new session_cookies.pkl file.
</commit_message>
<xml_diff>
--- a/crash_reports.xlsx
+++ b/crash_reports.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H32"/>
+  <dimension ref="A1:H52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -1358,6 +1358,550 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>1525066</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr"/>
+      <c r="C33" s="2" t="inlineStr"/>
+      <c r="D33" s="2" t="inlineStr"/>
+      <c r="E33" s="2" t="inlineStr"/>
+      <c r="F33" s="2" t="inlineStr"/>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 18:34:16</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>1525066</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>Accident Report</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>04/16/2026</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>04 / 16</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>add_shopping_cart
+Add to Cart
+Accident Report</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>DETROIT POLICE DEPARTMENT</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>FOUND</t>
+        </is>
+      </c>
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20 18:41:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>1525067</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>Accident Report</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>05/03/2026</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>05 / 03</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>add_shopping_cart
+Add to Cart
+Accident Report</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>DETROIT POLICE DEPARTMENT</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>FOUND</t>
+        </is>
+      </c>
+      <c r="H35" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20 18:43:32</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>1525068</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr"/>
+      <c r="C36" s="2" t="inlineStr"/>
+      <c r="D36" s="2" t="inlineStr"/>
+      <c r="E36" s="2" t="inlineStr"/>
+      <c r="F36" s="2" t="inlineStr"/>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 18:44:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>1525069</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr"/>
+      <c r="C37" s="2" t="inlineStr"/>
+      <c r="D37" s="2" t="inlineStr"/>
+      <c r="E37" s="2" t="inlineStr"/>
+      <c r="F37" s="2" t="inlineStr"/>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 18:46:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>1525070</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr"/>
+      <c r="C38" s="2" t="inlineStr"/>
+      <c r="D38" s="2" t="inlineStr"/>
+      <c r="E38" s="2" t="inlineStr"/>
+      <c r="F38" s="2" t="inlineStr"/>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 18:47:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>1525071</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr"/>
+      <c r="C39" s="2" t="inlineStr"/>
+      <c r="D39" s="2" t="inlineStr"/>
+      <c r="E39" s="2" t="inlineStr"/>
+      <c r="F39" s="2" t="inlineStr"/>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 18:48:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>1525066</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>Accident Report</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>S/B W OUTER DR / SANTA MARIA ST</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>MARRA L TISA GILL</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>DETROIT POLICE DEPARTMENT</t>
+        </is>
+      </c>
+      <c r="G40" s="3" t="inlineStr">
+        <is>
+          <t>FOUND</t>
+        </is>
+      </c>
+      <c r="H40" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20 18:51:33</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>1525067</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>Accident Report</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-03</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>PARK AVE / WASHINGTON BLVD</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>FAHR, SNELL</t>
+        </is>
+      </c>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>DETROIT POLICE DEPARTMENT</t>
+        </is>
+      </c>
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>FOUND</t>
+        </is>
+      </c>
+      <c r="H41" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20 18:51:49</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>1525068</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr"/>
+      <c r="C42" s="2" t="inlineStr"/>
+      <c r="D42" s="2" t="inlineStr"/>
+      <c r="E42" s="2" t="inlineStr"/>
+      <c r="F42" s="2" t="inlineStr"/>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 18:52:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>1525069</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr"/>
+      <c r="C43" s="2" t="inlineStr"/>
+      <c r="D43" s="2" t="inlineStr"/>
+      <c r="E43" s="2" t="inlineStr"/>
+      <c r="F43" s="2" t="inlineStr"/>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 18:53:10</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>1525070</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr"/>
+      <c r="C44" s="2" t="inlineStr"/>
+      <c r="D44" s="2" t="inlineStr"/>
+      <c r="E44" s="2" t="inlineStr"/>
+      <c r="F44" s="2" t="inlineStr"/>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 18:53:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>1525071</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr"/>
+      <c r="C45" s="2" t="inlineStr"/>
+      <c r="D45" s="2" t="inlineStr"/>
+      <c r="E45" s="2" t="inlineStr"/>
+      <c r="F45" s="2" t="inlineStr"/>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 18:54:18</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>1525072</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr"/>
+      <c r="C46" s="2" t="inlineStr"/>
+      <c r="D46" s="2" t="inlineStr"/>
+      <c r="E46" s="2" t="inlineStr"/>
+      <c r="F46" s="2" t="inlineStr"/>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 18:54:34</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>1525073</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr"/>
+      <c r="C47" s="2" t="inlineStr"/>
+      <c r="D47" s="2" t="inlineStr"/>
+      <c r="E47" s="2" t="inlineStr"/>
+      <c r="F47" s="2" t="inlineStr"/>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 18:54:50</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>1525074</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr"/>
+      <c r="C48" s="2" t="inlineStr"/>
+      <c r="D48" s="2" t="inlineStr"/>
+      <c r="E48" s="2" t="inlineStr"/>
+      <c r="F48" s="2" t="inlineStr"/>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 18:55:18</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>1525075</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr"/>
+      <c r="C49" s="2" t="inlineStr"/>
+      <c r="D49" s="2" t="inlineStr"/>
+      <c r="E49" s="2" t="inlineStr"/>
+      <c r="F49" s="2" t="inlineStr"/>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 18:55:34</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>1525076</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr"/>
+      <c r="C50" s="2" t="inlineStr"/>
+      <c r="D50" s="2" t="inlineStr"/>
+      <c r="E50" s="2" t="inlineStr"/>
+      <c r="F50" s="2" t="inlineStr"/>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 18:55:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>1525077</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr"/>
+      <c r="C51" s="2" t="inlineStr"/>
+      <c r="D51" s="2" t="inlineStr"/>
+      <c r="E51" s="2" t="inlineStr"/>
+      <c r="F51" s="2" t="inlineStr"/>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 18:56:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>1525078</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>Accident Report</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-21</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>S/B SOUTHFIELD SERV DR / HESSEL ST</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>MILES, SERVICES</t>
+        </is>
+      </c>
+      <c r="F52" s="3" t="inlineStr">
+        <is>
+          <t>DETROIT POLICE DEPARTMENT</t>
+        </is>
+      </c>
+      <c r="G52" s="3" t="inlineStr">
+        <is>
+          <t>FOUND</t>
+        </is>
+      </c>
+      <c r="H52" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20 18:56:52</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Switch to NO-LOGIN mode; remove account rotation
Change the scraper to use a NO-LOGIN (direct URL) session flow and remove account-rotation logic. main.py: drop account rotation and multi-account rate-limit handling, simplify output, and call run_search_session with no_login=True; keep progress saving and brief inter-batch pauses. searcher.py: add _get_session_no_login() to build a requests.Session from a headless browser visit, introduce pause/backoff schedules (_LIMIT_PAUSE_SCHEDULE, _MAX_LIMIT_CYCLES), and refactor run_search_session to support no_login mode — on SEARCH_LIMIT_REACHED it now performs dynamic pause cycles, refreshes the session, and will raise LIMIT_EXHAUSTED after exhausted cycles; legacy account-rotation paths are preserved but inactive. Update progress.txt (advance start number) and refresh crash_reports.xlsx.
</commit_message>
<xml_diff>
--- a/crash_reports.xlsx
+++ b/crash_reports.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H52"/>
+  <dimension ref="A1:H172"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -1902,6 +1902,3506 @@
         </is>
       </c>
     </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>1525066</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>Accident Report</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>S/B W OUTER DR / SANTA MARIA ST</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t>MARRA L TISA GILL</t>
+        </is>
+      </c>
+      <c r="F53" s="3" t="inlineStr">
+        <is>
+          <t>DETROIT POLICE DEPARTMENT</t>
+        </is>
+      </c>
+      <c r="G53" s="3" t="inlineStr">
+        <is>
+          <t>FOUND</t>
+        </is>
+      </c>
+      <c r="H53" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20 19:55:06</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t>1525066</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>Accident Report</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>S/B W OUTER DR / SANTA MARIA ST</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="inlineStr">
+        <is>
+          <t>MARRA L TISA GILL</t>
+        </is>
+      </c>
+      <c r="F54" s="3" t="inlineStr">
+        <is>
+          <t>DETROIT POLICE DEPARTMENT</t>
+        </is>
+      </c>
+      <c r="G54" s="3" t="inlineStr">
+        <is>
+          <t>FOUND</t>
+        </is>
+      </c>
+      <c r="H54" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20 19:55:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t>1525066</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>Accident Report</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>S/B W OUTER DR / SANTA MARIA ST</t>
+        </is>
+      </c>
+      <c r="E55" s="3" t="inlineStr">
+        <is>
+          <t>MARRA L TISA GILL</t>
+        </is>
+      </c>
+      <c r="F55" s="3" t="inlineStr">
+        <is>
+          <t>DETROIT POLICE DEPARTMENT</t>
+        </is>
+      </c>
+      <c r="G55" s="3" t="inlineStr">
+        <is>
+          <t>FOUND</t>
+        </is>
+      </c>
+      <c r="H55" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20 19:56:48</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="3" t="inlineStr">
+        <is>
+          <t>1525067</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>Accident Report</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-03</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>PARK AVE / WASHINGTON BLVD</t>
+        </is>
+      </c>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>FAHR, SNELL</t>
+        </is>
+      </c>
+      <c r="F56" s="3" t="inlineStr">
+        <is>
+          <t>DETROIT POLICE DEPARTMENT</t>
+        </is>
+      </c>
+      <c r="G56" s="3" t="inlineStr">
+        <is>
+          <t>FOUND</t>
+        </is>
+      </c>
+      <c r="H56" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20 19:57:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>1525068</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr"/>
+      <c r="C57" s="2" t="inlineStr"/>
+      <c r="D57" s="2" t="inlineStr"/>
+      <c r="E57" s="2" t="inlineStr"/>
+      <c r="F57" s="2" t="inlineStr"/>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 19:57:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>1525069</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr"/>
+      <c r="C58" s="2" t="inlineStr"/>
+      <c r="D58" s="2" t="inlineStr"/>
+      <c r="E58" s="2" t="inlineStr"/>
+      <c r="F58" s="2" t="inlineStr"/>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 19:57:35</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>1525070</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr"/>
+      <c r="C59" s="2" t="inlineStr"/>
+      <c r="D59" s="2" t="inlineStr"/>
+      <c r="E59" s="2" t="inlineStr"/>
+      <c r="F59" s="2" t="inlineStr"/>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 19:58:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>1525071</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr"/>
+      <c r="C60" s="2" t="inlineStr"/>
+      <c r="D60" s="2" t="inlineStr"/>
+      <c r="E60" s="2" t="inlineStr"/>
+      <c r="F60" s="2" t="inlineStr"/>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 19:58:44</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>1525072</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr"/>
+      <c r="C61" s="2" t="inlineStr"/>
+      <c r="D61" s="2" t="inlineStr"/>
+      <c r="E61" s="2" t="inlineStr"/>
+      <c r="F61" s="2" t="inlineStr"/>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 19:59:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>1525073</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr"/>
+      <c r="C62" s="2" t="inlineStr"/>
+      <c r="D62" s="2" t="inlineStr"/>
+      <c r="E62" s="2" t="inlineStr"/>
+      <c r="F62" s="2" t="inlineStr"/>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 19:59:16</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>1525074</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr"/>
+      <c r="C63" s="2" t="inlineStr"/>
+      <c r="D63" s="2" t="inlineStr"/>
+      <c r="E63" s="2" t="inlineStr"/>
+      <c r="F63" s="2" t="inlineStr"/>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H63" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 19:59:32</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>1525075</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr"/>
+      <c r="C64" s="2" t="inlineStr"/>
+      <c r="D64" s="2" t="inlineStr"/>
+      <c r="E64" s="2" t="inlineStr"/>
+      <c r="F64" s="2" t="inlineStr"/>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 19:59:48</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>1525076</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr"/>
+      <c r="C65" s="2" t="inlineStr"/>
+      <c r="D65" s="2" t="inlineStr"/>
+      <c r="E65" s="2" t="inlineStr"/>
+      <c r="F65" s="2" t="inlineStr"/>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 20:00:09</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>1525077</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr"/>
+      <c r="C66" s="2" t="inlineStr"/>
+      <c r="D66" s="2" t="inlineStr"/>
+      <c r="E66" s="2" t="inlineStr"/>
+      <c r="F66" s="2" t="inlineStr"/>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 20:00:25</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="3" t="inlineStr">
+        <is>
+          <t>1525078</t>
+        </is>
+      </c>
+      <c r="B67" s="3" t="inlineStr">
+        <is>
+          <t>Accident Report</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-21</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="inlineStr">
+        <is>
+          <t>S/B SOUTHFIELD SERV DR / HESSEL ST</t>
+        </is>
+      </c>
+      <c r="E67" s="3" t="inlineStr">
+        <is>
+          <t>MILES, SERVICES</t>
+        </is>
+      </c>
+      <c r="F67" s="3" t="inlineStr">
+        <is>
+          <t>DETROIT POLICE DEPARTMENT</t>
+        </is>
+      </c>
+      <c r="G67" s="3" t="inlineStr">
+        <is>
+          <t>FOUND</t>
+        </is>
+      </c>
+      <c r="H67" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20 20:00:41</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="3" t="inlineStr">
+        <is>
+          <t>1525066</t>
+        </is>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>Accident Report</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="inlineStr">
+        <is>
+          <t>S/B W OUTER DR / SANTA MARIA ST</t>
+        </is>
+      </c>
+      <c r="E68" s="3" t="inlineStr">
+        <is>
+          <t>MARRA L TISA GILL</t>
+        </is>
+      </c>
+      <c r="F68" s="3" t="inlineStr">
+        <is>
+          <t>DETROIT POLICE DEPARTMENT</t>
+        </is>
+      </c>
+      <c r="G68" s="3" t="inlineStr">
+        <is>
+          <t>FOUND</t>
+        </is>
+      </c>
+      <c r="H68" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20 20:42:18</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="3" t="inlineStr">
+        <is>
+          <t>1525067</t>
+        </is>
+      </c>
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t>Accident Report</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-03</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="inlineStr">
+        <is>
+          <t>PARK AVE / WASHINGTON BLVD</t>
+        </is>
+      </c>
+      <c r="E69" s="3" t="inlineStr">
+        <is>
+          <t>FAHR, SNELL</t>
+        </is>
+      </c>
+      <c r="F69" s="3" t="inlineStr">
+        <is>
+          <t>DETROIT POLICE DEPARTMENT</t>
+        </is>
+      </c>
+      <c r="G69" s="3" t="inlineStr">
+        <is>
+          <t>FOUND</t>
+        </is>
+      </c>
+      <c r="H69" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20 20:42:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>1525068</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr"/>
+      <c r="C70" s="2" t="inlineStr"/>
+      <c r="D70" s="2" t="inlineStr"/>
+      <c r="E70" s="2" t="inlineStr"/>
+      <c r="F70" s="2" t="inlineStr"/>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 20:44:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>1525069</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr"/>
+      <c r="C71" s="2" t="inlineStr"/>
+      <c r="D71" s="2" t="inlineStr"/>
+      <c r="E71" s="2" t="inlineStr"/>
+      <c r="F71" s="2" t="inlineStr"/>
+      <c r="G71" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H71" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 20:44:35</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>1525070</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr"/>
+      <c r="C72" s="2" t="inlineStr"/>
+      <c r="D72" s="2" t="inlineStr"/>
+      <c r="E72" s="2" t="inlineStr"/>
+      <c r="F72" s="2" t="inlineStr"/>
+      <c r="G72" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H72" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 20:46:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>1525071</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr"/>
+      <c r="C73" s="2" t="inlineStr"/>
+      <c r="D73" s="2" t="inlineStr"/>
+      <c r="E73" s="2" t="inlineStr"/>
+      <c r="F73" s="2" t="inlineStr"/>
+      <c r="G73" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H73" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 20:46:23</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>1525072</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr"/>
+      <c r="C74" s="2" t="inlineStr"/>
+      <c r="D74" s="2" t="inlineStr"/>
+      <c r="E74" s="2" t="inlineStr"/>
+      <c r="F74" s="2" t="inlineStr"/>
+      <c r="G74" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H74" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 20:46:39</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>1525073</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr"/>
+      <c r="C75" s="2" t="inlineStr"/>
+      <c r="D75" s="2" t="inlineStr"/>
+      <c r="E75" s="2" t="inlineStr"/>
+      <c r="F75" s="2" t="inlineStr"/>
+      <c r="G75" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H75" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 20:47:32</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>1525074</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr"/>
+      <c r="C76" s="2" t="inlineStr"/>
+      <c r="D76" s="2" t="inlineStr"/>
+      <c r="E76" s="2" t="inlineStr"/>
+      <c r="F76" s="2" t="inlineStr"/>
+      <c r="G76" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H76" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 20:47:48</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>1525075</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr"/>
+      <c r="C77" s="2" t="inlineStr"/>
+      <c r="D77" s="2" t="inlineStr"/>
+      <c r="E77" s="2" t="inlineStr"/>
+      <c r="F77" s="2" t="inlineStr"/>
+      <c r="G77" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H77" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 20:48:03</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>1525076</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr"/>
+      <c r="C78" s="2" t="inlineStr"/>
+      <c r="D78" s="2" t="inlineStr"/>
+      <c r="E78" s="2" t="inlineStr"/>
+      <c r="F78" s="2" t="inlineStr"/>
+      <c r="G78" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H78" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 20:48:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>1525077</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr"/>
+      <c r="C79" s="2" t="inlineStr"/>
+      <c r="D79" s="2" t="inlineStr"/>
+      <c r="E79" s="2" t="inlineStr"/>
+      <c r="F79" s="2" t="inlineStr"/>
+      <c r="G79" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H79" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 20:48:34</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>1525078</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr"/>
+      <c r="C80" s="2" t="inlineStr"/>
+      <c r="D80" s="2" t="inlineStr"/>
+      <c r="E80" s="2" t="inlineStr"/>
+      <c r="F80" s="2" t="inlineStr"/>
+      <c r="G80" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H80" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 20:48:50</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>1525079</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr"/>
+      <c r="C81" s="2" t="inlineStr"/>
+      <c r="D81" s="2" t="inlineStr"/>
+      <c r="E81" s="2" t="inlineStr"/>
+      <c r="F81" s="2" t="inlineStr"/>
+      <c r="G81" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H81" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 20:49:18</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>1525080</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr"/>
+      <c r="C82" s="2" t="inlineStr"/>
+      <c r="D82" s="2" t="inlineStr"/>
+      <c r="E82" s="2" t="inlineStr"/>
+      <c r="F82" s="2" t="inlineStr"/>
+      <c r="G82" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H82" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 20:49:34</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>1525081</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr"/>
+      <c r="C83" s="2" t="inlineStr"/>
+      <c r="D83" s="2" t="inlineStr"/>
+      <c r="E83" s="2" t="inlineStr"/>
+      <c r="F83" s="2" t="inlineStr"/>
+      <c r="G83" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H83" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 20:49:49</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>1525082</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr"/>
+      <c r="C84" s="2" t="inlineStr"/>
+      <c r="D84" s="2" t="inlineStr"/>
+      <c r="E84" s="2" t="inlineStr"/>
+      <c r="F84" s="2" t="inlineStr"/>
+      <c r="G84" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H84" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 20:50:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>1525083</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr"/>
+      <c r="C85" s="2" t="inlineStr"/>
+      <c r="D85" s="2" t="inlineStr"/>
+      <c r="E85" s="2" t="inlineStr"/>
+      <c r="F85" s="2" t="inlineStr"/>
+      <c r="G85" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H85" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 20:50:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>1525084</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr"/>
+      <c r="C86" s="2" t="inlineStr"/>
+      <c r="D86" s="2" t="inlineStr"/>
+      <c r="E86" s="2" t="inlineStr"/>
+      <c r="F86" s="2" t="inlineStr"/>
+      <c r="G86" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H86" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 20:51:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>1525085</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr"/>
+      <c r="C87" s="2" t="inlineStr"/>
+      <c r="D87" s="2" t="inlineStr"/>
+      <c r="E87" s="2" t="inlineStr"/>
+      <c r="F87" s="2" t="inlineStr"/>
+      <c r="G87" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H87" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 20:51:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>1525086</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr"/>
+      <c r="C88" s="2" t="inlineStr"/>
+      <c r="D88" s="2" t="inlineStr"/>
+      <c r="E88" s="2" t="inlineStr"/>
+      <c r="F88" s="2" t="inlineStr"/>
+      <c r="G88" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H88" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 20:51:50</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="3" t="inlineStr">
+        <is>
+          <t>1525066</t>
+        </is>
+      </c>
+      <c r="B89" s="3" t="inlineStr">
+        <is>
+          <t>Accident Report</t>
+        </is>
+      </c>
+      <c r="C89" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="inlineStr">
+        <is>
+          <t>S/B W OUTER DR / SANTA MARIA ST</t>
+        </is>
+      </c>
+      <c r="E89" s="3" t="inlineStr">
+        <is>
+          <t>MARRA L TISA GILL</t>
+        </is>
+      </c>
+      <c r="F89" s="3" t="inlineStr">
+        <is>
+          <t>DETROIT POLICE DEPARTMENT</t>
+        </is>
+      </c>
+      <c r="G89" s="3" t="inlineStr">
+        <is>
+          <t>FOUND</t>
+        </is>
+      </c>
+      <c r="H89" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20 21:52:53</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="3" t="inlineStr">
+        <is>
+          <t>1525067</t>
+        </is>
+      </c>
+      <c r="B90" s="3" t="inlineStr">
+        <is>
+          <t>Accident Report</t>
+        </is>
+      </c>
+      <c r="C90" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-03</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="inlineStr">
+        <is>
+          <t>PARK AVE / WASHINGTON BLVD</t>
+        </is>
+      </c>
+      <c r="E90" s="3" t="inlineStr">
+        <is>
+          <t>FAHR, SNELL</t>
+        </is>
+      </c>
+      <c r="F90" s="3" t="inlineStr">
+        <is>
+          <t>DETROIT POLICE DEPARTMENT</t>
+        </is>
+      </c>
+      <c r="G90" s="3" t="inlineStr">
+        <is>
+          <t>FOUND</t>
+        </is>
+      </c>
+      <c r="H90" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20 21:53:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>1525068</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr"/>
+      <c r="C91" s="2" t="inlineStr"/>
+      <c r="D91" s="2" t="inlineStr"/>
+      <c r="E91" s="2" t="inlineStr"/>
+      <c r="F91" s="2" t="inlineStr"/>
+      <c r="G91" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H91" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 21:54:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>1525069</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr"/>
+      <c r="C92" s="2" t="inlineStr"/>
+      <c r="D92" s="2" t="inlineStr"/>
+      <c r="E92" s="2" t="inlineStr"/>
+      <c r="F92" s="2" t="inlineStr"/>
+      <c r="G92" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H92" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 21:55:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>1525070</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="inlineStr"/>
+      <c r="C93" s="2" t="inlineStr"/>
+      <c r="D93" s="2" t="inlineStr"/>
+      <c r="E93" s="2" t="inlineStr"/>
+      <c r="F93" s="2" t="inlineStr"/>
+      <c r="G93" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H93" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 21:55:44</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>1525071</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="inlineStr"/>
+      <c r="C94" s="2" t="inlineStr"/>
+      <c r="D94" s="2" t="inlineStr"/>
+      <c r="E94" s="2" t="inlineStr"/>
+      <c r="F94" s="2" t="inlineStr"/>
+      <c r="G94" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H94" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 21:56:06</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>1525072</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="inlineStr"/>
+      <c r="C95" s="2" t="inlineStr"/>
+      <c r="D95" s="2" t="inlineStr"/>
+      <c r="E95" s="2" t="inlineStr"/>
+      <c r="F95" s="2" t="inlineStr"/>
+      <c r="G95" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H95" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 21:56:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>1525073</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr"/>
+      <c r="C96" s="2" t="inlineStr"/>
+      <c r="D96" s="2" t="inlineStr"/>
+      <c r="E96" s="2" t="inlineStr"/>
+      <c r="F96" s="2" t="inlineStr"/>
+      <c r="G96" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H96" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 21:56:52</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="3" t="inlineStr">
+        <is>
+          <t>1525066</t>
+        </is>
+      </c>
+      <c r="B97" s="3" t="inlineStr">
+        <is>
+          <t>Accident Report</t>
+        </is>
+      </c>
+      <c r="C97" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="inlineStr">
+        <is>
+          <t>S/B W OUTER DR / SANTA MARIA ST</t>
+        </is>
+      </c>
+      <c r="E97" s="3" t="inlineStr">
+        <is>
+          <t>MARRA L TISA GILL</t>
+        </is>
+      </c>
+      <c r="F97" s="3" t="inlineStr">
+        <is>
+          <t>DETROIT POLICE DEPARTMENT</t>
+        </is>
+      </c>
+      <c r="G97" s="3" t="inlineStr">
+        <is>
+          <t>FOUND</t>
+        </is>
+      </c>
+      <c r="H97" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20 22:11:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="3" t="inlineStr">
+        <is>
+          <t>1525067</t>
+        </is>
+      </c>
+      <c r="B98" s="3" t="inlineStr">
+        <is>
+          <t>Accident Report</t>
+        </is>
+      </c>
+      <c r="C98" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-03</t>
+        </is>
+      </c>
+      <c r="D98" s="3" t="inlineStr">
+        <is>
+          <t>PARK AVE / WASHINGTON BLVD</t>
+        </is>
+      </c>
+      <c r="E98" s="3" t="inlineStr">
+        <is>
+          <t>FAHR, SNELL</t>
+        </is>
+      </c>
+      <c r="F98" s="3" t="inlineStr">
+        <is>
+          <t>DETROIT POLICE DEPARTMENT</t>
+        </is>
+      </c>
+      <c r="G98" s="3" t="inlineStr">
+        <is>
+          <t>FOUND</t>
+        </is>
+      </c>
+      <c r="H98" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20 22:12:09</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="inlineStr">
+        <is>
+          <t>1525068</t>
+        </is>
+      </c>
+      <c r="B99" s="2" t="inlineStr"/>
+      <c r="C99" s="2" t="inlineStr"/>
+      <c r="D99" s="2" t="inlineStr"/>
+      <c r="E99" s="2" t="inlineStr"/>
+      <c r="F99" s="2" t="inlineStr"/>
+      <c r="G99" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H99" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 22:12:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>1525069</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="inlineStr"/>
+      <c r="C100" s="2" t="inlineStr"/>
+      <c r="D100" s="2" t="inlineStr"/>
+      <c r="E100" s="2" t="inlineStr"/>
+      <c r="F100" s="2" t="inlineStr"/>
+      <c r="G100" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H100" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 22:13:32</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>1525070</t>
+        </is>
+      </c>
+      <c r="B101" s="2" t="inlineStr"/>
+      <c r="C101" s="2" t="inlineStr"/>
+      <c r="D101" s="2" t="inlineStr"/>
+      <c r="E101" s="2" t="inlineStr"/>
+      <c r="F101" s="2" t="inlineStr"/>
+      <c r="G101" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H101" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 22:13:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>1525071</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="inlineStr"/>
+      <c r="C102" s="2" t="inlineStr"/>
+      <c r="D102" s="2" t="inlineStr"/>
+      <c r="E102" s="2" t="inlineStr"/>
+      <c r="F102" s="2" t="inlineStr"/>
+      <c r="G102" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H102" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 22:14:18</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>1525072</t>
+        </is>
+      </c>
+      <c r="B103" s="2" t="inlineStr"/>
+      <c r="C103" s="2" t="inlineStr"/>
+      <c r="D103" s="2" t="inlineStr"/>
+      <c r="E103" s="2" t="inlineStr"/>
+      <c r="F103" s="2" t="inlineStr"/>
+      <c r="G103" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H103" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 22:15:39</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>1525073</t>
+        </is>
+      </c>
+      <c r="B104" s="2" t="inlineStr"/>
+      <c r="C104" s="2" t="inlineStr"/>
+      <c r="D104" s="2" t="inlineStr"/>
+      <c r="E104" s="2" t="inlineStr"/>
+      <c r="F104" s="2" t="inlineStr"/>
+      <c r="G104" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H104" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 22:16:16</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>1525074</t>
+        </is>
+      </c>
+      <c r="B105" s="2" t="inlineStr"/>
+      <c r="C105" s="2" t="inlineStr"/>
+      <c r="D105" s="2" t="inlineStr"/>
+      <c r="E105" s="2" t="inlineStr"/>
+      <c r="F105" s="2" t="inlineStr"/>
+      <c r="G105" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H105" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 22:16:39</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>1525075</t>
+        </is>
+      </c>
+      <c r="B106" s="2" t="inlineStr"/>
+      <c r="C106" s="2" t="inlineStr"/>
+      <c r="D106" s="2" t="inlineStr"/>
+      <c r="E106" s="2" t="inlineStr"/>
+      <c r="F106" s="2" t="inlineStr"/>
+      <c r="G106" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H106" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 22:17:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>1525076</t>
+        </is>
+      </c>
+      <c r="B107" s="2" t="inlineStr"/>
+      <c r="C107" s="2" t="inlineStr"/>
+      <c r="D107" s="2" t="inlineStr"/>
+      <c r="E107" s="2" t="inlineStr"/>
+      <c r="F107" s="2" t="inlineStr"/>
+      <c r="G107" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H107" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 22:21:22</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>1525077</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr"/>
+      <c r="C108" s="2" t="inlineStr"/>
+      <c r="D108" s="2" t="inlineStr"/>
+      <c r="E108" s="2" t="inlineStr"/>
+      <c r="F108" s="2" t="inlineStr"/>
+      <c r="G108" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H108" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 22:21:46</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="3" t="inlineStr">
+        <is>
+          <t>1525078</t>
+        </is>
+      </c>
+      <c r="B109" s="3" t="inlineStr">
+        <is>
+          <t>Accident Report</t>
+        </is>
+      </c>
+      <c r="C109" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-21</t>
+        </is>
+      </c>
+      <c r="D109" s="3" t="inlineStr">
+        <is>
+          <t>S/B SOUTHFIELD SERV DR / HESSEL ST</t>
+        </is>
+      </c>
+      <c r="E109" s="3" t="inlineStr">
+        <is>
+          <t>MILES, SERVICES</t>
+        </is>
+      </c>
+      <c r="F109" s="3" t="inlineStr">
+        <is>
+          <t>DETROIT POLICE DEPARTMENT</t>
+        </is>
+      </c>
+      <c r="G109" s="3" t="inlineStr">
+        <is>
+          <t>FOUND</t>
+        </is>
+      </c>
+      <c r="H109" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20 22:22:09</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="3" t="inlineStr">
+        <is>
+          <t>1525079</t>
+        </is>
+      </c>
+      <c r="B110" s="3" t="inlineStr">
+        <is>
+          <t>Accident Report</t>
+        </is>
+      </c>
+      <c r="C110" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="D110" s="3" t="inlineStr">
+        <is>
+          <t>MACK AVE / FAIRVIEW ST</t>
+        </is>
+      </c>
+      <c r="E110" s="3" t="inlineStr">
+        <is>
+          <t>JONES, JONES, MASON, WAGNER</t>
+        </is>
+      </c>
+      <c r="F110" s="3" t="inlineStr">
+        <is>
+          <t>DETROIT POLICE DEPARTMENT</t>
+        </is>
+      </c>
+      <c r="G110" s="3" t="inlineStr">
+        <is>
+          <t>FOUND</t>
+        </is>
+      </c>
+      <c r="H110" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20 22:23:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="3" t="inlineStr">
+        <is>
+          <t>1525080</t>
+        </is>
+      </c>
+      <c r="B111" s="3" t="inlineStr">
+        <is>
+          <t>Accident Report</t>
+        </is>
+      </c>
+      <c r="C111" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="D111" s="3" t="inlineStr">
+        <is>
+          <t>FISHER FWY / BRUSH ST</t>
+        </is>
+      </c>
+      <c r="E111" s="3" t="inlineStr">
+        <is>
+          <t>SCHNEIDER</t>
+        </is>
+      </c>
+      <c r="F111" s="3" t="inlineStr">
+        <is>
+          <t>DETROIT POLICE DEPARTMENT</t>
+        </is>
+      </c>
+      <c r="G111" s="3" t="inlineStr">
+        <is>
+          <t>FOUND</t>
+        </is>
+      </c>
+      <c r="H111" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20 22:23:53</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="3" t="inlineStr">
+        <is>
+          <t>1525081</t>
+        </is>
+      </c>
+      <c r="B112" s="3" t="inlineStr">
+        <is>
+          <t>Accident Report</t>
+        </is>
+      </c>
+      <c r="C112" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="D112" s="3" t="inlineStr">
+        <is>
+          <t>W EDSEL FORD SERVICE DR / 30TH ST</t>
+        </is>
+      </c>
+      <c r="E112" s="3" t="inlineStr">
+        <is>
+          <t>BARRON, LLOYD, MONTEIRO REA</t>
+        </is>
+      </c>
+      <c r="F112" s="3" t="inlineStr">
+        <is>
+          <t>DETROIT POLICE DEPARTMENT</t>
+        </is>
+      </c>
+      <c r="G112" s="3" t="inlineStr">
+        <is>
+          <t>FOUND</t>
+        </is>
+      </c>
+      <c r="H112" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20 22:24:41</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="3" t="inlineStr">
+        <is>
+          <t>1525082</t>
+        </is>
+      </c>
+      <c r="B113" s="3" t="inlineStr">
+        <is>
+          <t>Accident Report</t>
+        </is>
+      </c>
+      <c r="C113" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="D113" s="3" t="inlineStr">
+        <is>
+          <t>51ST ST / SAINT STEPHENS ST</t>
+        </is>
+      </c>
+      <c r="E113" s="3" t="inlineStr">
+        <is>
+          <t>BOYER, SMITH</t>
+        </is>
+      </c>
+      <c r="F113" s="3" t="inlineStr">
+        <is>
+          <t>DETROIT POLICE DEPARTMENT</t>
+        </is>
+      </c>
+      <c r="G113" s="3" t="inlineStr">
+        <is>
+          <t>FOUND</t>
+        </is>
+      </c>
+      <c r="H113" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20 22:25:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="inlineStr">
+        <is>
+          <t>1525083</t>
+        </is>
+      </c>
+      <c r="B114" s="2" t="inlineStr"/>
+      <c r="C114" s="2" t="inlineStr"/>
+      <c r="D114" s="2" t="inlineStr"/>
+      <c r="E114" s="2" t="inlineStr"/>
+      <c r="F114" s="2" t="inlineStr"/>
+      <c r="G114" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H114" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 22:25:52</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="2" t="inlineStr">
+        <is>
+          <t>1525084</t>
+        </is>
+      </c>
+      <c r="B115" s="2" t="inlineStr"/>
+      <c r="C115" s="2" t="inlineStr"/>
+      <c r="D115" s="2" t="inlineStr"/>
+      <c r="E115" s="2" t="inlineStr"/>
+      <c r="F115" s="2" t="inlineStr"/>
+      <c r="G115" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H115" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 22:26:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="inlineStr">
+        <is>
+          <t>1525085</t>
+        </is>
+      </c>
+      <c r="B116" s="2" t="inlineStr"/>
+      <c r="C116" s="2" t="inlineStr"/>
+      <c r="D116" s="2" t="inlineStr"/>
+      <c r="E116" s="2" t="inlineStr"/>
+      <c r="F116" s="2" t="inlineStr"/>
+      <c r="G116" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H116" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 22:27:03</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="2" t="inlineStr">
+        <is>
+          <t>1525086</t>
+        </is>
+      </c>
+      <c r="B117" s="2" t="inlineStr"/>
+      <c r="C117" s="2" t="inlineStr"/>
+      <c r="D117" s="2" t="inlineStr"/>
+      <c r="E117" s="2" t="inlineStr"/>
+      <c r="F117" s="2" t="inlineStr"/>
+      <c r="G117" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H117" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 22:27:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="inlineStr">
+        <is>
+          <t>1525087</t>
+        </is>
+      </c>
+      <c r="B118" s="2" t="inlineStr"/>
+      <c r="C118" s="2" t="inlineStr"/>
+      <c r="D118" s="2" t="inlineStr"/>
+      <c r="E118" s="2" t="inlineStr"/>
+      <c r="F118" s="2" t="inlineStr"/>
+      <c r="G118" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H118" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 22:27:53</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="2" t="inlineStr">
+        <is>
+          <t>1525088</t>
+        </is>
+      </c>
+      <c r="B119" s="2" t="inlineStr"/>
+      <c r="C119" s="2" t="inlineStr"/>
+      <c r="D119" s="2" t="inlineStr"/>
+      <c r="E119" s="2" t="inlineStr"/>
+      <c r="F119" s="2" t="inlineStr"/>
+      <c r="G119" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H119" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 22:28:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="2" t="inlineStr">
+        <is>
+          <t>1525089</t>
+        </is>
+      </c>
+      <c r="B120" s="2" t="inlineStr"/>
+      <c r="C120" s="2" t="inlineStr"/>
+      <c r="D120" s="2" t="inlineStr"/>
+      <c r="E120" s="2" t="inlineStr"/>
+      <c r="F120" s="2" t="inlineStr"/>
+      <c r="G120" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H120" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 22:28:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="3" t="inlineStr">
+        <is>
+          <t>1525090</t>
+        </is>
+      </c>
+      <c r="B121" s="3" t="inlineStr">
+        <is>
+          <t>Accident Report</t>
+        </is>
+      </c>
+      <c r="C121" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="D121" s="3" t="inlineStr">
+        <is>
+          <t>SCHAEFER HWY / GROVE ST</t>
+        </is>
+      </c>
+      <c r="E121" s="3" t="inlineStr">
+        <is>
+          <t>HARDY, HARRIS, MASON HARDY</t>
+        </is>
+      </c>
+      <c r="F121" s="3" t="inlineStr">
+        <is>
+          <t>DETROIT POLICE DEPARTMENT</t>
+        </is>
+      </c>
+      <c r="G121" s="3" t="inlineStr">
+        <is>
+          <t>FOUND</t>
+        </is>
+      </c>
+      <c r="H121" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20 22:29:26</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="3" t="inlineStr">
+        <is>
+          <t>1525091</t>
+        </is>
+      </c>
+      <c r="B122" s="3" t="inlineStr">
+        <is>
+          <t>Accident Report</t>
+        </is>
+      </c>
+      <c r="C122" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="D122" s="3" t="inlineStr">
+        <is>
+          <t>7 MILE RD  RD / ANCHESTER</t>
+        </is>
+      </c>
+      <c r="E122" s="3" t="inlineStr">
+        <is>
+          <t>DIALLO, HARPER, KENNEDY</t>
+        </is>
+      </c>
+      <c r="F122" s="3" t="inlineStr">
+        <is>
+          <t>DETROIT POLICE DEPARTMENT</t>
+        </is>
+      </c>
+      <c r="G122" s="3" t="inlineStr">
+        <is>
+          <t>FOUND</t>
+        </is>
+      </c>
+      <c r="H122" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20 22:29:49</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="3" t="inlineStr">
+        <is>
+          <t>1525092</t>
+        </is>
+      </c>
+      <c r="B123" s="3" t="inlineStr">
+        <is>
+          <t>Accident Report</t>
+        </is>
+      </c>
+      <c r="C123" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="D123" s="3" t="inlineStr">
+        <is>
+          <t>I-75 SOUTH FREEWAY / ROSA PARKS BLVD</t>
+        </is>
+      </c>
+      <c r="E123" s="3" t="inlineStr">
+        <is>
+          <t>STACHERSKI, STACHERSKI</t>
+        </is>
+      </c>
+      <c r="F123" s="3" t="inlineStr">
+        <is>
+          <t>DETROIT POLICE DEPARTMENT</t>
+        </is>
+      </c>
+      <c r="G123" s="3" t="inlineStr">
+        <is>
+          <t>FOUND</t>
+        </is>
+      </c>
+      <c r="H123" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20 22:30:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="inlineStr">
+        <is>
+          <t>1525093</t>
+        </is>
+      </c>
+      <c r="B124" s="2" t="inlineStr"/>
+      <c r="C124" s="2" t="inlineStr"/>
+      <c r="D124" s="2" t="inlineStr"/>
+      <c r="E124" s="2" t="inlineStr"/>
+      <c r="F124" s="2" t="inlineStr"/>
+      <c r="G124" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H124" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 22:30:35</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="2" t="inlineStr">
+        <is>
+          <t>1525094</t>
+        </is>
+      </c>
+      <c r="B125" s="2" t="inlineStr"/>
+      <c r="C125" s="2" t="inlineStr"/>
+      <c r="D125" s="2" t="inlineStr"/>
+      <c r="E125" s="2" t="inlineStr"/>
+      <c r="F125" s="2" t="inlineStr"/>
+      <c r="G125" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H125" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 22:30:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="3" t="inlineStr">
+        <is>
+          <t>1525095</t>
+        </is>
+      </c>
+      <c r="B126" s="3" t="inlineStr">
+        <is>
+          <t>Accident Report</t>
+        </is>
+      </c>
+      <c r="C126" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="D126" s="3" t="inlineStr">
+        <is>
+          <t>HOUSTON WHITTIER AVE / HAYES ST</t>
+        </is>
+      </c>
+      <c r="E126" s="3" t="inlineStr">
+        <is>
+          <t>JONES</t>
+        </is>
+      </c>
+      <c r="F126" s="3" t="inlineStr">
+        <is>
+          <t>DETROIT POLICE DEPARTMENT</t>
+        </is>
+      </c>
+      <c r="G126" s="3" t="inlineStr">
+        <is>
+          <t>FOUND</t>
+        </is>
+      </c>
+      <c r="H126" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20 22:31:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="3" t="inlineStr">
+        <is>
+          <t>1525066</t>
+        </is>
+      </c>
+      <c r="B127" s="3" t="inlineStr">
+        <is>
+          <t>Accident Report</t>
+        </is>
+      </c>
+      <c r="C127" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="D127" s="3" t="inlineStr">
+        <is>
+          <t>S/B W OUTER DR / SANTA MARIA ST</t>
+        </is>
+      </c>
+      <c r="E127" s="3" t="inlineStr">
+        <is>
+          <t>MARRA L TISA GILL</t>
+        </is>
+      </c>
+      <c r="F127" s="3" t="inlineStr">
+        <is>
+          <t>DETROIT POLICE DEPARTMENT</t>
+        </is>
+      </c>
+      <c r="G127" s="3" t="inlineStr">
+        <is>
+          <t>FOUND</t>
+        </is>
+      </c>
+      <c r="H127" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20 22:55:53</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="3" t="inlineStr">
+        <is>
+          <t>1525067</t>
+        </is>
+      </c>
+      <c r="B128" s="3" t="inlineStr">
+        <is>
+          <t>Accident Report</t>
+        </is>
+      </c>
+      <c r="C128" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-03</t>
+        </is>
+      </c>
+      <c r="D128" s="3" t="inlineStr">
+        <is>
+          <t>PARK AVE / WASHINGTON BLVD</t>
+        </is>
+      </c>
+      <c r="E128" s="3" t="inlineStr">
+        <is>
+          <t>FAHR, SNELL</t>
+        </is>
+      </c>
+      <c r="F128" s="3" t="inlineStr">
+        <is>
+          <t>DETROIT POLICE DEPARTMENT</t>
+        </is>
+      </c>
+      <c r="G128" s="3" t="inlineStr">
+        <is>
+          <t>FOUND</t>
+        </is>
+      </c>
+      <c r="H128" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20 22:56:17</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="2" t="inlineStr">
+        <is>
+          <t>1525068</t>
+        </is>
+      </c>
+      <c r="B129" s="2" t="inlineStr"/>
+      <c r="C129" s="2" t="inlineStr"/>
+      <c r="D129" s="2" t="inlineStr"/>
+      <c r="E129" s="2" t="inlineStr"/>
+      <c r="F129" s="2" t="inlineStr"/>
+      <c r="G129" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H129" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20 22:57:31</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="3" t="inlineStr">
+        <is>
+          <t>1525066</t>
+        </is>
+      </c>
+      <c r="B130" s="3" t="inlineStr">
+        <is>
+          <t>Accident Report</t>
+        </is>
+      </c>
+      <c r="C130" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="D130" s="3" t="inlineStr">
+        <is>
+          <t>S/B W OUTER DR / SANTA MARIA ST</t>
+        </is>
+      </c>
+      <c r="E130" s="3" t="inlineStr">
+        <is>
+          <t>MARRA L TISA GILL</t>
+        </is>
+      </c>
+      <c r="F130" s="3" t="inlineStr">
+        <is>
+          <t>DETROIT POLICE DEPARTMENT</t>
+        </is>
+      </c>
+      <c r="G130" s="3" t="inlineStr">
+        <is>
+          <t>FOUND</t>
+        </is>
+      </c>
+      <c r="H130" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-21 00:16:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="3" t="inlineStr">
+        <is>
+          <t>1525067</t>
+        </is>
+      </c>
+      <c r="B131" s="3" t="inlineStr">
+        <is>
+          <t>Accident Report</t>
+        </is>
+      </c>
+      <c r="C131" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-03</t>
+        </is>
+      </c>
+      <c r="D131" s="3" t="inlineStr">
+        <is>
+          <t>PARK AVE / WASHINGTON BLVD</t>
+        </is>
+      </c>
+      <c r="E131" s="3" t="inlineStr">
+        <is>
+          <t>FAHR, SNELL</t>
+        </is>
+      </c>
+      <c r="F131" s="3" t="inlineStr">
+        <is>
+          <t>DETROIT POLICE DEPARTMENT</t>
+        </is>
+      </c>
+      <c r="G131" s="3" t="inlineStr">
+        <is>
+          <t>FOUND</t>
+        </is>
+      </c>
+      <c r="H131" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-21 00:16:25</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="2" t="inlineStr">
+        <is>
+          <t>1525068</t>
+        </is>
+      </c>
+      <c r="B132" s="2" t="inlineStr"/>
+      <c r="C132" s="2" t="inlineStr"/>
+      <c r="D132" s="2" t="inlineStr"/>
+      <c r="E132" s="2" t="inlineStr"/>
+      <c r="F132" s="2" t="inlineStr"/>
+      <c r="G132" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H132" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21 00:17:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="3" t="inlineStr">
+        <is>
+          <t>1525066</t>
+        </is>
+      </c>
+      <c r="B133" s="3" t="inlineStr">
+        <is>
+          <t>Accident Report</t>
+        </is>
+      </c>
+      <c r="C133" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="D133" s="3" t="inlineStr">
+        <is>
+          <t>S/B W OUTER DR / SANTA MARIA ST</t>
+        </is>
+      </c>
+      <c r="E133" s="3" t="inlineStr">
+        <is>
+          <t>MARRA L TISA GILL</t>
+        </is>
+      </c>
+      <c r="F133" s="3" t="inlineStr">
+        <is>
+          <t>DETROIT POLICE DEPARTMENT</t>
+        </is>
+      </c>
+      <c r="G133" s="3" t="inlineStr">
+        <is>
+          <t>FOUND</t>
+        </is>
+      </c>
+      <c r="H133" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-21 01:22:52</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="3" t="inlineStr">
+        <is>
+          <t>1525067</t>
+        </is>
+      </c>
+      <c r="B134" s="3" t="inlineStr">
+        <is>
+          <t>Accident Report</t>
+        </is>
+      </c>
+      <c r="C134" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-03</t>
+        </is>
+      </c>
+      <c r="D134" s="3" t="inlineStr">
+        <is>
+          <t>PARK AVE / WASHINGTON BLVD</t>
+        </is>
+      </c>
+      <c r="E134" s="3" t="inlineStr">
+        <is>
+          <t>FAHR, SNELL</t>
+        </is>
+      </c>
+      <c r="F134" s="3" t="inlineStr">
+        <is>
+          <t>DETROIT POLICE DEPARTMENT</t>
+        </is>
+      </c>
+      <c r="G134" s="3" t="inlineStr">
+        <is>
+          <t>FOUND</t>
+        </is>
+      </c>
+      <c r="H134" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-21 01:24:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="2" t="inlineStr">
+        <is>
+          <t>1525068</t>
+        </is>
+      </c>
+      <c r="B135" s="2" t="inlineStr"/>
+      <c r="C135" s="2" t="inlineStr"/>
+      <c r="D135" s="2" t="inlineStr"/>
+      <c r="E135" s="2" t="inlineStr"/>
+      <c r="F135" s="2" t="inlineStr"/>
+      <c r="G135" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H135" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21 01:26:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="2" t="inlineStr">
+        <is>
+          <t>1525069</t>
+        </is>
+      </c>
+      <c r="B136" s="2" t="inlineStr"/>
+      <c r="C136" s="2" t="inlineStr"/>
+      <c r="D136" s="2" t="inlineStr"/>
+      <c r="E136" s="2" t="inlineStr"/>
+      <c r="F136" s="2" t="inlineStr"/>
+      <c r="G136" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H136" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21 01:27:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="2" t="inlineStr">
+        <is>
+          <t>1525070</t>
+        </is>
+      </c>
+      <c r="B137" s="2" t="inlineStr"/>
+      <c r="C137" s="2" t="inlineStr"/>
+      <c r="D137" s="2" t="inlineStr"/>
+      <c r="E137" s="2" t="inlineStr"/>
+      <c r="F137" s="2" t="inlineStr"/>
+      <c r="G137" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H137" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21 01:28:03</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="2" t="inlineStr">
+        <is>
+          <t>1525071</t>
+        </is>
+      </c>
+      <c r="B138" s="2" t="inlineStr"/>
+      <c r="C138" s="2" t="inlineStr"/>
+      <c r="D138" s="2" t="inlineStr"/>
+      <c r="E138" s="2" t="inlineStr"/>
+      <c r="F138" s="2" t="inlineStr"/>
+      <c r="G138" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H138" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21 01:29:17</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="2" t="inlineStr">
+        <is>
+          <t>1525072</t>
+        </is>
+      </c>
+      <c r="B139" s="2" t="inlineStr"/>
+      <c r="C139" s="2" t="inlineStr"/>
+      <c r="D139" s="2" t="inlineStr"/>
+      <c r="E139" s="2" t="inlineStr"/>
+      <c r="F139" s="2" t="inlineStr"/>
+      <c r="G139" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H139" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21 01:30:06</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="inlineStr">
+        <is>
+          <t>1525073</t>
+        </is>
+      </c>
+      <c r="B140" s="2" t="inlineStr"/>
+      <c r="C140" s="2" t="inlineStr"/>
+      <c r="D140" s="2" t="inlineStr"/>
+      <c r="E140" s="2" t="inlineStr"/>
+      <c r="F140" s="2" t="inlineStr"/>
+      <c r="G140" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H140" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21 01:30:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="2" t="inlineStr">
+        <is>
+          <t>1525074</t>
+        </is>
+      </c>
+      <c r="B141" s="2" t="inlineStr"/>
+      <c r="C141" s="2" t="inlineStr"/>
+      <c r="D141" s="2" t="inlineStr"/>
+      <c r="E141" s="2" t="inlineStr"/>
+      <c r="F141" s="2" t="inlineStr"/>
+      <c r="G141" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H141" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21 01:30:51</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="2" t="inlineStr">
+        <is>
+          <t>1525075</t>
+        </is>
+      </c>
+      <c r="B142" s="2" t="inlineStr"/>
+      <c r="C142" s="2" t="inlineStr"/>
+      <c r="D142" s="2" t="inlineStr"/>
+      <c r="E142" s="2" t="inlineStr"/>
+      <c r="F142" s="2" t="inlineStr"/>
+      <c r="G142" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H142" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21 01:31:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="2" t="inlineStr">
+        <is>
+          <t>1525076</t>
+        </is>
+      </c>
+      <c r="B143" s="2" t="inlineStr"/>
+      <c r="C143" s="2" t="inlineStr"/>
+      <c r="D143" s="2" t="inlineStr"/>
+      <c r="E143" s="2" t="inlineStr"/>
+      <c r="F143" s="2" t="inlineStr"/>
+      <c r="G143" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H143" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21 01:31:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="2" t="inlineStr">
+        <is>
+          <t>1525077</t>
+        </is>
+      </c>
+      <c r="B144" s="2" t="inlineStr"/>
+      <c r="C144" s="2" t="inlineStr"/>
+      <c r="D144" s="2" t="inlineStr"/>
+      <c r="E144" s="2" t="inlineStr"/>
+      <c r="F144" s="2" t="inlineStr"/>
+      <c r="G144" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H144" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21 01:32:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="3" t="inlineStr">
+        <is>
+          <t>1525078</t>
+        </is>
+      </c>
+      <c r="B145" s="3" t="inlineStr">
+        <is>
+          <t>Accident Report</t>
+        </is>
+      </c>
+      <c r="C145" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-21</t>
+        </is>
+      </c>
+      <c r="D145" s="3" t="inlineStr">
+        <is>
+          <t>S/B SOUTHFIELD SERV DR / HESSEL ST</t>
+        </is>
+      </c>
+      <c r="E145" s="3" t="inlineStr">
+        <is>
+          <t>MILES, SERVICES</t>
+        </is>
+      </c>
+      <c r="F145" s="3" t="inlineStr">
+        <is>
+          <t>DETROIT POLICE DEPARTMENT</t>
+        </is>
+      </c>
+      <c r="G145" s="3" t="inlineStr">
+        <is>
+          <t>FOUND</t>
+        </is>
+      </c>
+      <c r="H145" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-21 01:32:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="3" t="inlineStr">
+        <is>
+          <t>1525079</t>
+        </is>
+      </c>
+      <c r="B146" s="3" t="inlineStr">
+        <is>
+          <t>Accident Report</t>
+        </is>
+      </c>
+      <c r="C146" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="D146" s="3" t="inlineStr">
+        <is>
+          <t>MACK AVE / FAIRVIEW ST</t>
+        </is>
+      </c>
+      <c r="E146" s="3" t="inlineStr">
+        <is>
+          <t>JONES, JONES, MASON, WAGNER</t>
+        </is>
+      </c>
+      <c r="F146" s="3" t="inlineStr">
+        <is>
+          <t>DETROIT POLICE DEPARTMENT</t>
+        </is>
+      </c>
+      <c r="G146" s="3" t="inlineStr">
+        <is>
+          <t>FOUND</t>
+        </is>
+      </c>
+      <c r="H146" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-21 01:33:18</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="3" t="inlineStr">
+        <is>
+          <t>1525080</t>
+        </is>
+      </c>
+      <c r="B147" s="3" t="inlineStr">
+        <is>
+          <t>Accident Report</t>
+        </is>
+      </c>
+      <c r="C147" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="D147" s="3" t="inlineStr">
+        <is>
+          <t>FISHER FWY / BRUSH ST</t>
+        </is>
+      </c>
+      <c r="E147" s="3" t="inlineStr">
+        <is>
+          <t>SCHNEIDER</t>
+        </is>
+      </c>
+      <c r="F147" s="3" t="inlineStr">
+        <is>
+          <t>DETROIT POLICE DEPARTMENT</t>
+        </is>
+      </c>
+      <c r="G147" s="3" t="inlineStr">
+        <is>
+          <t>FOUND</t>
+        </is>
+      </c>
+      <c r="H147" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-21 01:33:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="3" t="inlineStr">
+        <is>
+          <t>1525081</t>
+        </is>
+      </c>
+      <c r="B148" s="3" t="inlineStr">
+        <is>
+          <t>Accident Report</t>
+        </is>
+      </c>
+      <c r="C148" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="D148" s="3" t="inlineStr">
+        <is>
+          <t>W EDSEL FORD SERVICE DR / 30TH ST</t>
+        </is>
+      </c>
+      <c r="E148" s="3" t="inlineStr">
+        <is>
+          <t>BARRON, LLOYD, MONTEIRO REA</t>
+        </is>
+      </c>
+      <c r="F148" s="3" t="inlineStr">
+        <is>
+          <t>DETROIT POLICE DEPARTMENT</t>
+        </is>
+      </c>
+      <c r="G148" s="3" t="inlineStr">
+        <is>
+          <t>FOUND</t>
+        </is>
+      </c>
+      <c r="H148" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-21 01:34:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="3" t="inlineStr">
+        <is>
+          <t>1525082</t>
+        </is>
+      </c>
+      <c r="B149" s="3" t="inlineStr">
+        <is>
+          <t>Accident Report</t>
+        </is>
+      </c>
+      <c r="C149" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="D149" s="3" t="inlineStr">
+        <is>
+          <t>51ST ST / SAINT STEPHENS ST</t>
+        </is>
+      </c>
+      <c r="E149" s="3" t="inlineStr">
+        <is>
+          <t>BOYER, SMITH</t>
+        </is>
+      </c>
+      <c r="F149" s="3" t="inlineStr">
+        <is>
+          <t>DETROIT POLICE DEPARTMENT</t>
+        </is>
+      </c>
+      <c r="G149" s="3" t="inlineStr">
+        <is>
+          <t>FOUND</t>
+        </is>
+      </c>
+      <c r="H149" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-21 01:34:51</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="2" t="inlineStr">
+        <is>
+          <t>1525083</t>
+        </is>
+      </c>
+      <c r="B150" s="2" t="inlineStr"/>
+      <c r="C150" s="2" t="inlineStr"/>
+      <c r="D150" s="2" t="inlineStr"/>
+      <c r="E150" s="2" t="inlineStr"/>
+      <c r="F150" s="2" t="inlineStr"/>
+      <c r="G150" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H150" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21 01:35:13</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="2" t="inlineStr">
+        <is>
+          <t>1525084</t>
+        </is>
+      </c>
+      <c r="B151" s="2" t="inlineStr"/>
+      <c r="C151" s="2" t="inlineStr"/>
+      <c r="D151" s="2" t="inlineStr"/>
+      <c r="E151" s="2" t="inlineStr"/>
+      <c r="F151" s="2" t="inlineStr"/>
+      <c r="G151" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H151" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21 01:35:36</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="inlineStr">
+        <is>
+          <t>1525085</t>
+        </is>
+      </c>
+      <c r="B152" s="2" t="inlineStr"/>
+      <c r="C152" s="2" t="inlineStr"/>
+      <c r="D152" s="2" t="inlineStr"/>
+      <c r="E152" s="2" t="inlineStr"/>
+      <c r="F152" s="2" t="inlineStr"/>
+      <c r="G152" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H152" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21 02:10:33</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="2" t="inlineStr">
+        <is>
+          <t>1525086</t>
+        </is>
+      </c>
+      <c r="B153" s="2" t="inlineStr"/>
+      <c r="C153" s="2" t="inlineStr"/>
+      <c r="D153" s="2" t="inlineStr"/>
+      <c r="E153" s="2" t="inlineStr"/>
+      <c r="F153" s="2" t="inlineStr"/>
+      <c r="G153" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H153" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21 02:12:09</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="2" t="inlineStr">
+        <is>
+          <t>1525087</t>
+        </is>
+      </c>
+      <c r="B154" s="2" t="inlineStr"/>
+      <c r="C154" s="2" t="inlineStr"/>
+      <c r="D154" s="2" t="inlineStr"/>
+      <c r="E154" s="2" t="inlineStr"/>
+      <c r="F154" s="2" t="inlineStr"/>
+      <c r="G154" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H154" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21 02:12:33</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="2" t="inlineStr">
+        <is>
+          <t>1525088</t>
+        </is>
+      </c>
+      <c r="B155" s="2" t="inlineStr"/>
+      <c r="C155" s="2" t="inlineStr"/>
+      <c r="D155" s="2" t="inlineStr"/>
+      <c r="E155" s="2" t="inlineStr"/>
+      <c r="F155" s="2" t="inlineStr"/>
+      <c r="G155" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H155" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21 02:12:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="2" t="inlineStr">
+        <is>
+          <t>1525089</t>
+        </is>
+      </c>
+      <c r="B156" s="2" t="inlineStr"/>
+      <c r="C156" s="2" t="inlineStr"/>
+      <c r="D156" s="2" t="inlineStr"/>
+      <c r="E156" s="2" t="inlineStr"/>
+      <c r="F156" s="2" t="inlineStr"/>
+      <c r="G156" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H156" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21 02:13:18</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="3" t="inlineStr">
+        <is>
+          <t>1525090</t>
+        </is>
+      </c>
+      <c r="B157" s="3" t="inlineStr">
+        <is>
+          <t>Accident Report</t>
+        </is>
+      </c>
+      <c r="C157" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="D157" s="3" t="inlineStr">
+        <is>
+          <t>SCHAEFER HWY / GROVE ST</t>
+        </is>
+      </c>
+      <c r="E157" s="3" t="inlineStr">
+        <is>
+          <t>HARDY, HARRIS, MASON HARDY</t>
+        </is>
+      </c>
+      <c r="F157" s="3" t="inlineStr">
+        <is>
+          <t>DETROIT POLICE DEPARTMENT</t>
+        </is>
+      </c>
+      <c r="G157" s="3" t="inlineStr">
+        <is>
+          <t>FOUND</t>
+        </is>
+      </c>
+      <c r="H157" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-21 02:13:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="3" t="inlineStr">
+        <is>
+          <t>1525091</t>
+        </is>
+      </c>
+      <c r="B158" s="3" t="inlineStr">
+        <is>
+          <t>Accident Report</t>
+        </is>
+      </c>
+      <c r="C158" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="D158" s="3" t="inlineStr">
+        <is>
+          <t>7 MILE RD  RD / ANCHESTER</t>
+        </is>
+      </c>
+      <c r="E158" s="3" t="inlineStr">
+        <is>
+          <t>DIALLO, HARPER, KENNEDY</t>
+        </is>
+      </c>
+      <c r="F158" s="3" t="inlineStr">
+        <is>
+          <t>DETROIT POLICE DEPARTMENT</t>
+        </is>
+      </c>
+      <c r="G158" s="3" t="inlineStr">
+        <is>
+          <t>FOUND</t>
+        </is>
+      </c>
+      <c r="H158" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-21 02:14:17</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="3" t="inlineStr">
+        <is>
+          <t>1525092</t>
+        </is>
+      </c>
+      <c r="B159" s="3" t="inlineStr">
+        <is>
+          <t>Accident Report</t>
+        </is>
+      </c>
+      <c r="C159" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="D159" s="3" t="inlineStr">
+        <is>
+          <t>I-75 SOUTH FREEWAY / ROSA PARKS BLVD</t>
+        </is>
+      </c>
+      <c r="E159" s="3" t="inlineStr">
+        <is>
+          <t>STACHERSKI, STACHERSKI</t>
+        </is>
+      </c>
+      <c r="F159" s="3" t="inlineStr">
+        <is>
+          <t>DETROIT POLICE DEPARTMENT</t>
+        </is>
+      </c>
+      <c r="G159" s="3" t="inlineStr">
+        <is>
+          <t>FOUND</t>
+        </is>
+      </c>
+      <c r="H159" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-21 02:14:39</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="2" t="inlineStr">
+        <is>
+          <t>1525093</t>
+        </is>
+      </c>
+      <c r="B160" s="2" t="inlineStr"/>
+      <c r="C160" s="2" t="inlineStr"/>
+      <c r="D160" s="2" t="inlineStr"/>
+      <c r="E160" s="2" t="inlineStr"/>
+      <c r="F160" s="2" t="inlineStr"/>
+      <c r="G160" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H160" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21 02:15:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="2" t="inlineStr">
+        <is>
+          <t>1525094</t>
+        </is>
+      </c>
+      <c r="B161" s="2" t="inlineStr"/>
+      <c r="C161" s="2" t="inlineStr"/>
+      <c r="D161" s="2" t="inlineStr"/>
+      <c r="E161" s="2" t="inlineStr"/>
+      <c r="F161" s="2" t="inlineStr"/>
+      <c r="G161" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H161" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21 02:15:25</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="3" t="inlineStr">
+        <is>
+          <t>1525095</t>
+        </is>
+      </c>
+      <c r="B162" s="3" t="inlineStr">
+        <is>
+          <t>Accident Report</t>
+        </is>
+      </c>
+      <c r="C162" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="D162" s="3" t="inlineStr">
+        <is>
+          <t>HOUSTON WHITTIER AVE / HAYES ST</t>
+        </is>
+      </c>
+      <c r="E162" s="3" t="inlineStr">
+        <is>
+          <t>JONES</t>
+        </is>
+      </c>
+      <c r="F162" s="3" t="inlineStr">
+        <is>
+          <t>DETROIT POLICE DEPARTMENT</t>
+        </is>
+      </c>
+      <c r="G162" s="3" t="inlineStr">
+        <is>
+          <t>FOUND</t>
+        </is>
+      </c>
+      <c r="H162" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-21 02:15:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="3" t="inlineStr">
+        <is>
+          <t>1525096</t>
+        </is>
+      </c>
+      <c r="B163" s="3" t="inlineStr">
+        <is>
+          <t>Accident Report</t>
+        </is>
+      </c>
+      <c r="C163" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="D163" s="3" t="inlineStr">
+        <is>
+          <t>S/B GLASTON BURY AVE / MARGARETA ST</t>
+        </is>
+      </c>
+      <c r="E163" s="3" t="inlineStr">
+        <is>
+          <t>HUTCHINSON, LLC</t>
+        </is>
+      </c>
+      <c r="F163" s="3" t="inlineStr">
+        <is>
+          <t>DETROIT POLICE DEPARTMENT</t>
+        </is>
+      </c>
+      <c r="G163" s="3" t="inlineStr">
+        <is>
+          <t>FOUND</t>
+        </is>
+      </c>
+      <c r="H163" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-21 02:16:31</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="3" t="inlineStr">
+        <is>
+          <t>1525097</t>
+        </is>
+      </c>
+      <c r="B164" s="3" t="inlineStr">
+        <is>
+          <t>Accident Report</t>
+        </is>
+      </c>
+      <c r="C164" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="D164" s="3" t="inlineStr">
+        <is>
+          <t>TELEGRAPH / MCNICHOLS</t>
+        </is>
+      </c>
+      <c r="E164" s="3" t="inlineStr">
+        <is>
+          <t>LOCH</t>
+        </is>
+      </c>
+      <c r="F164" s="3" t="inlineStr">
+        <is>
+          <t>DETROIT POLICE DEPARTMENT</t>
+        </is>
+      </c>
+      <c r="G164" s="3" t="inlineStr">
+        <is>
+          <t>FOUND</t>
+        </is>
+      </c>
+      <c r="H164" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-21 02:16:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="3" t="inlineStr">
+        <is>
+          <t>1525098</t>
+        </is>
+      </c>
+      <c r="B165" s="3" t="inlineStr">
+        <is>
+          <t>Accident Report</t>
+        </is>
+      </c>
+      <c r="C165" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="D165" s="3" t="inlineStr">
+        <is>
+          <t>WYOMING / LYNDON ST</t>
+        </is>
+      </c>
+      <c r="E165" s="3" t="inlineStr">
+        <is>
+          <t>JACKSON, WILLIAMS</t>
+        </is>
+      </c>
+      <c r="F165" s="3" t="inlineStr">
+        <is>
+          <t>DETROIT POLICE DEPARTMENT</t>
+        </is>
+      </c>
+      <c r="G165" s="3" t="inlineStr">
+        <is>
+          <t>FOUND</t>
+        </is>
+      </c>
+      <c r="H165" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-21 02:17:16</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="2" t="inlineStr">
+        <is>
+          <t>1525099</t>
+        </is>
+      </c>
+      <c r="B166" s="2" t="inlineStr"/>
+      <c r="C166" s="2" t="inlineStr"/>
+      <c r="D166" s="2" t="inlineStr"/>
+      <c r="E166" s="2" t="inlineStr"/>
+      <c r="F166" s="2" t="inlineStr"/>
+      <c r="G166" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H166" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21 02:17:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="3" t="inlineStr">
+        <is>
+          <t>1525100</t>
+        </is>
+      </c>
+      <c r="B167" s="3" t="inlineStr">
+        <is>
+          <t>Accident Report</t>
+        </is>
+      </c>
+      <c r="C167" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="D167" s="3" t="inlineStr">
+        <is>
+          <t>E 8 MILE RD / TERRELL ST</t>
+        </is>
+      </c>
+      <c r="E167" s="3" t="inlineStr">
+        <is>
+          <t>CURB, KHAN</t>
+        </is>
+      </c>
+      <c r="F167" s="3" t="inlineStr">
+        <is>
+          <t>DETROIT POLICE DEPARTMENT</t>
+        </is>
+      </c>
+      <c r="G167" s="3" t="inlineStr">
+        <is>
+          <t>FOUND</t>
+        </is>
+      </c>
+      <c r="H167" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-21 02:18:03</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="2" t="inlineStr">
+        <is>
+          <t>1525101</t>
+        </is>
+      </c>
+      <c r="B168" s="2" t="inlineStr"/>
+      <c r="C168" s="2" t="inlineStr"/>
+      <c r="D168" s="2" t="inlineStr"/>
+      <c r="E168" s="2" t="inlineStr"/>
+      <c r="F168" s="2" t="inlineStr"/>
+      <c r="G168" s="2" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H168" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21 02:18:26</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="3" t="inlineStr">
+        <is>
+          <t>1525102</t>
+        </is>
+      </c>
+      <c r="B169" s="3" t="inlineStr">
+        <is>
+          <t>Accident Report</t>
+        </is>
+      </c>
+      <c r="C169" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="D169" s="3" t="inlineStr">
+        <is>
+          <t>E FOREST AVE / DEQUINDRE ST</t>
+        </is>
+      </c>
+      <c r="E169" s="3" t="inlineStr">
+        <is>
+          <t>BORUM, JEFFERSON, WILHELM</t>
+        </is>
+      </c>
+      <c r="F169" s="3" t="inlineStr">
+        <is>
+          <t>DETROIT POLICE DEPARTMENT</t>
+        </is>
+      </c>
+      <c r="G169" s="3" t="inlineStr">
+        <is>
+          <t>FOUND</t>
+        </is>
+      </c>
+      <c r="H169" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-21 02:18:49</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="3" t="inlineStr">
+        <is>
+          <t>1525103</t>
+        </is>
+      </c>
+      <c r="B170" s="3" t="inlineStr">
+        <is>
+          <t>Accident Report</t>
+        </is>
+      </c>
+      <c r="C170" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="D170" s="3" t="inlineStr">
+        <is>
+          <t>LAHSER RD / PEMBROKE AVE</t>
+        </is>
+      </c>
+      <c r="E170" s="3" t="inlineStr">
+        <is>
+          <t>TARVER</t>
+        </is>
+      </c>
+      <c r="F170" s="3" t="inlineStr">
+        <is>
+          <t>DETROIT POLICE DEPARTMENT</t>
+        </is>
+      </c>
+      <c r="G170" s="3" t="inlineStr">
+        <is>
+          <t>FOUND</t>
+        </is>
+      </c>
+      <c r="H170" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-21 02:19:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="3" t="inlineStr">
+        <is>
+          <t>1525104</t>
+        </is>
+      </c>
+      <c r="B171" s="3" t="inlineStr">
+        <is>
+          <t>Accident Report</t>
+        </is>
+      </c>
+      <c r="C171" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-19</t>
+        </is>
+      </c>
+      <c r="D171" s="3" t="inlineStr">
+        <is>
+          <t>MITCHELL / E 7 MILE</t>
+        </is>
+      </c>
+      <c r="E171" s="3" t="inlineStr">
+        <is>
+          <t>HILL, JOHNSON, MAXWELL</t>
+        </is>
+      </c>
+      <c r="F171" s="3" t="inlineStr">
+        <is>
+          <t>DETROIT POLICE DEPARTMENT</t>
+        </is>
+      </c>
+      <c r="G171" s="3" t="inlineStr">
+        <is>
+          <t>FOUND</t>
+        </is>
+      </c>
+      <c r="H171" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-21 02:19:34</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="3" t="inlineStr">
+        <is>
+          <t>1525066</t>
+        </is>
+      </c>
+      <c r="B172" s="3" t="inlineStr">
+        <is>
+          <t>Accident Report</t>
+        </is>
+      </c>
+      <c r="C172" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="D172" s="3" t="inlineStr">
+        <is>
+          <t>S/B W OUTER DR / SANTA MARIA ST</t>
+        </is>
+      </c>
+      <c r="E172" s="3" t="inlineStr">
+        <is>
+          <t>MARRA L TISA GILL</t>
+        </is>
+      </c>
+      <c r="F172" s="3" t="inlineStr">
+        <is>
+          <t>DETROIT POLICE DEPARTMENT</t>
+        </is>
+      </c>
+      <c r="G172" s="3" t="inlineStr">
+        <is>
+          <t>FOUND</t>
+        </is>
+      </c>
+      <c r="H172" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-21 03:30:09</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>